<commit_message>
Update soccer trades 2026-08-14 12:03:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Bundesliga/trades.xlsx
+++ b/data/sxbet/ligas/Bundesliga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+          <t>0x2d42370b05751a34d03be1367afb327b6e72ae3b341fa63651c557748608e06f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,15 +539,19 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>23.34</t>
+          <t>91.41</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4638</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786682534</t>
+          <t>1786706976</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>50.328841</t>
+          <t>168.110345</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,102 +643,2318 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0x078ea10216f3741d1757134ccf5904d995bb1b31fb4dda2433595eacd7c26ca8</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.5425</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1786705939</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>6.635945</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0x89225b7389497635b7a6d5762e0312ef71ce7e6aad4bacb31d914cb8e8063156</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>228.48997</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.8613</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xe385ab4b9eeee1b6ee91ce4a2452c903e1102819fc6a3ef47b0b71ecca4789e7</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1786704847</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>265.300401</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x798a2a121340304c054e489a82c2fbcbbacbb2b5a10fac5eccae9d0e6f953242</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>36.96</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1786704771</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>49.28</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0xd7c7ed5aee6d42691c0cdba24cc2a4844a2148619b251e896e222af12c3f399a</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>36.96</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1786704503</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>49.28</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0x91957fcc3f4e1390d64a84f24cad4ac44f2f9926c17ed7cd978de77f93ab840a</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>36.96</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786704472</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>49.28</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x33ec03964bc9b5353ad6c834080797ae574d6738a2f6ecafd9040ba4d9dc21d6</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>36.96</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786704050</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>49.28</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x060bae1553ca0b1b27e0303f5cb0b1a208018b22ad43c47887b7eab9174eb11f</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x1EEc232fcA954D560922A46C0dc77A1d5Fc1278C</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1.49999</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.7588</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786700992</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1.976923</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x89945f48362d177a1a075c347f0cee9e0d2949251232062e79954c3fdbda8548</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>36.69</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.7475</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786697954</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>49.083612</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0x93f8ae4db5435f2088469fb82cd900c151ecf6b1707f1fa749e6f328a01576ca</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>35.77998</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786696250</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>47.70664</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x6c37a9cb7783035c2363518b021ca262c492e837d2f5566a7197ec81c9c7de3c</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0x2Bd56fa0D7b1Add3639Ee23f32A2947576924f15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>557.83</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.5437</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786696222</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1025.894253</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0xb8844dc9cad239dda58468ea8057a5d42a49adaeb39f853d1d8a2f72f86b2a27</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22.83999</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.5437</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786695902</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>42.004579</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>0x54732df74313495ae4750f10f2ec1b1437622f274d00a56e3a61e0c23a1acde2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>296.6897</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.4612</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786695873</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>643.229702</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0x6388d0dbf04f19becbc0ad458a4000da4d11cf0c26aa897bddfdef754fa335a6</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>346.54</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786695869</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>641.740741</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x1d90dd2b57deb4a163be22ec0027c40ec930edc46ca3efc1b7765006d5e9eebe</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786695799</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>1.851852</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x48c4a72e45740310d60b3a648deeb512824e451ea186d1e82f9627f5d1bccd51</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0.99999</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786695700</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>1.33332</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0x4ebc4769fdeafa179bcff07b1f83a83c2f713dd0b038325187723d036f03b296</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0x9E555D159D333EAE7346aE58D3d57dDE9680a9F7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>484.79999</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786695653</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>897.777759</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0xb62e61543153c0b9ab6a1a3fd388b5a709ce3356240d5f06b0b8a0c62bad8b1a</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786695037</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0xcb685b4fae14c825bf9607310b4cfb4892294304396aedd620dbe8ca7410b54c</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1786694953</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>0xbd2bb212ebdbf36503fd81ffa846a8c770a6aae66b0380af0fcc4a45aa66cc55</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1786694900</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>23.34</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.4638</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1786682534</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>50.328841</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>0xbc3f9a4aae23f8578c48b6575d84b3634a2c81e75a2b7c12b7aa17d431671a0e</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
         <is>
           <t>2.08</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>1.2625</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Under/Over (2)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
         <is>
           <t>Bundesliga</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>LASK Linz vs SV Ried</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>LASK Linz</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>SV Ried</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>L19722986</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
         <is>
           <t>1786678003</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>1786728600</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>7.92381</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-14 13:04:43 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Bundesliga/trades.xlsx
+++ b/data/sxbet/ligas/Bundesliga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x2d42370b05751a34d03be1367afb327b6e72ae3b341fa63651c557748608e06f</t>
+          <t>0xd55646b617b0f28d4b7c8f4a7157567db85abf92b455bd498870f96fbaeb125a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>91.41</t>
+          <t>1.76999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>LASK Linz -0.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x8ed613eccc85721e5128096540f9355a0f8cf59e645c356e533ccd8eb1928ec5</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786706976</t>
+          <t>1786712107</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>168.110345</t>
+          <t>2.681803</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x078ea10216f3741d1757134ccf5904d995bb1b31fb4dda2433595eacd7c26ca8</t>
+          <t>0xc63dfc3e1f7d71137952fe723ef12e4c36bed56f14b5b69b20f56f7c04cb9fb1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>2515.19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786705939</t>
+          <t>1786711888</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6.635945</t>
+          <t>4625.636782</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,31 +755,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x89225b7389497635b7a6d5762e0312ef71ce7e6aad4bacb31d914cb8e8063156</t>
+          <t>0x2bcb64c2bfd3514856c15034bf37585fb056e6d201e48aa560646e765f2bf612</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>228.48997</t>
+          <t>26.12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.8613</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -802,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xe385ab4b9eeee1b6ee91ce4a2452c903e1102819fc6a3ef47b0b71ecca4789e7</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786704847</t>
+          <t>1786710267</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>265.300401</t>
+          <t>48.258661</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +867,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x798a2a121340304c054e489a82c2fbcbbacbb2b5a10fac5eccae9d0e6f953242</t>
+          <t>0xbc037195afbbb894f93552f09a96dbf26e085b032162fd371bdcd6e507cc6030</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -874,22 +882,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>22.3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -914,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786704771</t>
+          <t>1786709725</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>41.011494</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +979,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xd7c7ed5aee6d42691c0cdba24cc2a4844a2148619b251e896e222af12c3f399a</t>
+          <t>0x8bb6ce50f9cdd747617cc6ddd8923bac84c636a43b5747ece36118588d661e56</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,22 +994,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.6612</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -0.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1026,7 +1034,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x8ed613eccc85721e5128096540f9355a0f8cf59e645c356e533ccd8eb1928ec5</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786704503</t>
+          <t>1786709683</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>3.493384</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1091,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x91957fcc3f4e1390d64a84f24cad4ac44f2f9926c17ed7cd978de77f93ab840a</t>
+          <t>0x2d42370b05751a34d03be1367afb327b6e72ae3b341fa63651c557748608e06f</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,22 +1106,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>91.41</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1138,7 +1146,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1168,7 +1176,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786704472</t>
+          <t>1786706976</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1186,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>168.110345</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1203,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x33ec03964bc9b5353ad6c834080797ae574d6738a2f6ecafd9040ba4d9dc21d6</t>
+          <t>0x078ea10216f3741d1757134ccf5904d995bb1b31fb4dda2433595eacd7c26ca8</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1210,22 +1218,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1250,7 +1258,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1280,7 +1288,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786704050</t>
+          <t>1786705939</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1290,7 +1298,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>6.635945</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1307,39 +1315,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x060bae1553ca0b1b27e0303f5cb0b1a208018b22ad43c47887b7eab9174eb11f</t>
+          <t>0x89225b7389497635b7a6d5762e0312ef71ce7e6aad4bacb31d914cb8e8063156</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x1EEc232fcA954D560922A46C0dc77A1d5Fc1278C</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.49999</t>
+          <t>228.48997</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.7588</t>
+          <t>1.8613</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0xe385ab4b9eeee1b6ee91ce4a2452c903e1102819fc6a3ef47b0b71ecca4789e7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786700992</t>
+          <t>1786704847</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.976923</t>
+          <t>265.300401</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x89945f48362d177a1a075c347f0cee9e0d2949251232062e79954c3fdbda8548</t>
+          <t>0x798a2a121340304c054e489a82c2fbcbbacbb2b5a10fac5eccae9d0e6f953242</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1434,12 +1434,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>36.69</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.7475</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786697954</t>
+          <t>1786704771</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>49.083612</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1531,7 +1531,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x93f8ae4db5435f2088469fb82cd900c151ecf6b1707f1fa749e6f328a01576ca</t>
+          <t>0xd7c7ed5aee6d42691c0cdba24cc2a4844a2148619b251e896e222af12c3f399a</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>35.77998</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786696250</t>
+          <t>1786704503</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>47.70664</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1643,12 +1643,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x6c37a9cb7783035c2363518b021ca262c492e837d2f5566a7197ec81c9c7de3c</t>
+          <t>0x91957fcc3f4e1390d64a84f24cad4ac44f2f9926c17ed7cd978de77f93ab840a</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x2Bd56fa0D7b1Add3639Ee23f32A2947576924f15</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1658,22 +1658,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>557.83</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786696222</t>
+          <t>1786704472</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1025.894253</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1755,12 +1755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xb8844dc9cad239dda58468ea8057a5d42a49adaeb39f853d1d8a2f72f86b2a27</t>
+          <t>0x33ec03964bc9b5353ad6c834080797ae574d6738a2f6ecafd9040ba4d9dc21d6</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1770,22 +1770,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>22.83999</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786695902</t>
+          <t>1786704050</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>42.004579</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1867,31 +1867,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x54732df74313495ae4750f10f2ec1b1437622f274d00a56e3a61e0c23a1acde2</t>
+          <t>0x060bae1553ca0b1b27e0303f5cb0b1a208018b22ad43c47887b7eab9174eb11f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>0x1EEc232fcA954D560922A46C0dc77A1d5Fc1278C</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>296.6897</t>
+          <t>1.49999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.4612</t>
+          <t>1.7588</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -1914,7 +1922,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1944,7 +1952,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786695873</t>
+          <t>1786700992</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1954,7 +1962,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>643.229702</t>
+          <t>1.976923</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1971,12 +1979,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x6388d0dbf04f19becbc0ad458a4000da4d11cf0c26aa897bddfdef754fa335a6</t>
+          <t>0x89945f48362d177a1a075c347f0cee9e0d2949251232062e79954c3fdbda8548</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1986,22 +1994,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>346.54</t>
+          <t>36.69</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.7475</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2026,7 +2034,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2056,7 +2064,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786695869</t>
+          <t>1786697954</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2066,7 +2074,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>641.740741</t>
+          <t>49.083612</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2083,12 +2091,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x1d90dd2b57deb4a163be22ec0027c40ec930edc46ca3efc1b7765006d5e9eebe</t>
+          <t>0x93f8ae4db5435f2088469fb82cd900c151ecf6b1707f1fa749e6f328a01576ca</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2098,22 +2106,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>35.77998</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2138,7 +2146,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2168,7 +2176,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786695799</t>
+          <t>1786696250</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2178,7 +2186,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.851852</t>
+          <t>47.70664</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2195,12 +2203,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x48c4a72e45740310d60b3a648deeb512824e451ea186d1e82f9627f5d1bccd51</t>
+          <t>0x6c37a9cb7783035c2363518b021ca262c492e837d2f5566a7197ec81c9c7de3c</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x2Bd56fa0D7b1Add3639Ee23f32A2947576924f15</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2210,22 +2218,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>557.83</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2250,7 +2258,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2280,7 +2288,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786695700</t>
+          <t>1786696222</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2290,7 +2298,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.33332</t>
+          <t>1025.894253</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2307,12 +2315,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x4ebc4769fdeafa179bcff07b1f83a83c2f713dd0b038325187723d036f03b296</t>
+          <t>0xb8844dc9cad239dda58468ea8057a5d42a49adaeb39f853d1d8a2f72f86b2a27</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x9E555D159D333EAE7346aE58D3d57dDE9680a9F7</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2322,12 +2330,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>484.79999</t>
+          <t>22.83999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2392,7 +2400,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786695653</t>
+          <t>1786695902</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2402,7 +2410,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>897.777759</t>
+          <t>42.004579</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2419,27 +2427,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xb62e61543153c0b9ab6a1a3fd388b5a709ce3356240d5f06b0b8a0c62bad8b1a</t>
+          <t>0x54732df74313495ae4750f10f2ec1b1437622f274d00a56e3a61e0c23a1acde2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>296.6897</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.4612</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2447,11 +2451,7 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>LASK Linz -1</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786695037</t>
+          <t>1786695873</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>643.229702</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2531,12 +2531,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xcb685b4fae14c825bf9607310b4cfb4892294304396aedd620dbe8ca7410b54c</t>
+          <t>0x6388d0dbf04f19becbc0ad458a4000da4d11cf0c26aa897bddfdef754fa335a6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>346.54</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786694953</t>
+          <t>1786695869</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>641.740741</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2643,12 +2643,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xbd2bb212ebdbf36503fd81ffa846a8c770a6aae66b0380af0fcc4a45aa66cc55</t>
+          <t>0x1d90dd2b57deb4a163be22ec0027c40ec930edc46ca3efc1b7765006d5e9eebe</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786694900</t>
+          <t>1786695799</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>1.851852</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2755,31 +2755,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+          <t>0x48c4a72e45740310d60b3a648deeb512824e451ea186d1e82f9627f5d1bccd51</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>23.34</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.4638</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -2802,7 +2810,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2832,7 +2840,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786682534</t>
+          <t>1786695700</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2842,7 +2850,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>50.328841</t>
+          <t>1.33332</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2859,102 +2867,654 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>0x4ebc4769fdeafa179bcff07b1f83a83c2f713dd0b038325187723d036f03b296</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0x9E555D159D333EAE7346aE58D3d57dDE9680a9F7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>484.79999</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1786695653</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>897.777759</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0xb62e61543153c0b9ab6a1a3fd388b5a709ce3356240d5f06b0b8a0c62bad8b1a</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786695037</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0xcb685b4fae14c825bf9607310b4cfb4892294304396aedd620dbe8ca7410b54c</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1786694953</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0xbd2bb212ebdbf36503fd81ffa846a8c770a6aae66b0380af0fcc4a45aa66cc55</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786694900</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>23.34</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.4638</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786682534</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>50.328841</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>0xbc3f9a4aae23f8578c48b6575d84b3634a2c81e75a2b7c12b7aa17d431671a0e</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>2.08</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>1.2625</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Under/Over (2)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
         <is>
           <t>Bundesliga</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>LASK Linz vs SV Ried</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>LASK Linz</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>SV Ried</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>L19722986</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
         <is>
           <t>1786678003</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="S28" t="inlineStr">
         <is>
           <t>1786728600</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="T28" t="inlineStr">
         <is>
           <t>7.92381</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-14 15:04:33 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Bundesliga/trades.xlsx
+++ b/data/sxbet/ligas/Bundesliga/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:V32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xd55646b617b0f28d4b7c8f4a7157567db85abf92b455bd498870f96fbaeb125a</t>
+          <t>0x54c3e231f8760e93b735c3aad70b0f6d9bf290f79601bb3e545369171a42f0a6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.76999</t>
+          <t>26.06999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>1.5475</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Asian Handicap (-0.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LASK Linz -0.5</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x8ed613eccc85721e5128096540f9355a0f8cf59e645c356e533ccd8eb1928ec5</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786712107</t>
+          <t>1786716750</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.681803</t>
+          <t>47.61642</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xc63dfc3e1f7d71137952fe723ef12e4c36bed56f14b5b69b20f56f7c04cb9fb1</t>
+          <t>0x0221ccc43787d77e6f9bc6e244999aa02abe58f4c73f1e3e86f8c053ab060c42</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2515.19</t>
+          <t>66.68</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.495</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0xd395255f1fdaa1f3bea5a106e2055834680bdee9a58a41895c7a38f31f80beae</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786711888</t>
+          <t>1786714580</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>4625.636782</t>
+          <t>134.707071</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x2bcb64c2bfd3514856c15034bf37585fb056e6d201e48aa560646e765f2bf612</t>
+          <t>0xa45e722b2f8857d69d73317ce3084dc2e69df0903bf371409451731203c676d2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -763,31 +763,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>26.12</t>
+          <t>30.68</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5413</t>
+          <t>1.625</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>LASK Linz -1</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -810,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x154b733171c7f01e7789a18e341fb6e3e8121f02e74e4febf14af52e6bd870fc</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786710267</t>
+          <t>1786714022</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>48.258661</t>
+          <t>49.088</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xbc037195afbbb894f93552f09a96dbf26e085b032162fd371bdcd6e507cc6030</t>
+          <t>0x8c91335ae9ec2badc857e675d35ff8e3818eb0b802c3d05fc3ebf796c3f18195</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,22 +874,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22.3</t>
+          <t>6.89</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4937</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -922,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0xd395255f1fdaa1f3bea5a106e2055834680bdee9a58a41895c7a38f31f80beae</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786709725</t>
+          <t>1786713936</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>41.011494</t>
+          <t>13.95443</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x8bb6ce50f9cdd747617cc6ddd8923bac84c636a43b5747ece36118588d661e56</t>
+          <t>0xd55646b617b0f28d4b7c8f4a7157567db85abf92b455bd498870f96fbaeb125a</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -994,12 +986,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.31</t>
+          <t>1.76999</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.6612</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1064,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786709683</t>
+          <t>1786712107</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>3.493384</t>
+          <t>2.681803</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,12 +1083,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2d42370b05751a34d03be1367afb327b6e72ae3b341fa63651c557748608e06f</t>
+          <t>0xc63dfc3e1f7d71137952fe723ef12e4c36bed56f14b5b69b20f56f7c04cb9fb1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1106,7 +1098,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>91.41</t>
+          <t>2515.19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1176,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786706976</t>
+          <t>1786711888</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1186,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>168.110345</t>
+          <t>4625.636782</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1203,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x078ea10216f3741d1757134ccf5904d995bb1b31fb4dda2433595eacd7c26ca8</t>
+          <t>0x2bcb64c2bfd3514856c15034bf37585fb056e6d201e48aa560646e765f2bf612</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1218,12 +1210,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>26.12</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5425</t>
+          <t>1.5413</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1288,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786705939</t>
+          <t>1786710267</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1298,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6.635945</t>
+          <t>48.258661</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1315,31 +1307,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x89225b7389497635b7a6d5762e0312ef71ce7e6aad4bacb31d914cb8e8063156</t>
+          <t>0xbc037195afbbb894f93552f09a96dbf26e085b032162fd371bdcd6e507cc6030</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>228.48997</t>
+          <t>22.3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.8613</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xe385ab4b9eeee1b6ee91ce4a2452c903e1102819fc6a3ef47b0b71ecca4789e7</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786704847</t>
+          <t>1786709725</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>265.300401</t>
+          <t>41.011494</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1419,7 +1419,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x798a2a121340304c054e489a82c2fbcbbacbb2b5a10fac5eccae9d0e6f953242</t>
+          <t>0x8bb6ce50f9cdd747617cc6ddd8923bac84c636a43b5747ece36118588d661e56</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1434,22 +1434,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.6612</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-0.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -0.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x8ed613eccc85721e5128096540f9355a0f8cf59e645c356e533ccd8eb1928ec5</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786704771</t>
+          <t>1786709683</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>3.493384</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1531,12 +1531,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xd7c7ed5aee6d42691c0cdba24cc2a4844a2148619b251e896e222af12c3f399a</t>
+          <t>0x2d42370b05751a34d03be1367afb327b6e72ae3b341fa63651c557748608e06f</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1546,22 +1546,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>91.41</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786704503</t>
+          <t>1786706976</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>168.110345</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1643,7 +1643,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x91957fcc3f4e1390d64a84f24cad4ac44f2f9926c17ed7cd978de77f93ab840a</t>
+          <t>0x078ea10216f3741d1757134ccf5904d995bb1b31fb4dda2433595eacd7c26ca8</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1658,22 +1658,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5425</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786704472</t>
+          <t>1786705939</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>6.635945</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1755,39 +1755,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x33ec03964bc9b5353ad6c834080797ae574d6738a2f6ecafd9040ba4d9dc21d6</t>
+          <t>0x89225b7389497635b7a6d5762e0312ef71ce7e6aad4bacb31d914cb8e8063156</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>36.96</t>
+          <t>228.48997</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.8613</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -1810,7 +1802,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0xe385ab4b9eeee1b6ee91ce4a2452c903e1102819fc6a3ef47b0b71ecca4789e7</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1840,7 +1832,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786704050</t>
+          <t>1786704847</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1850,7 +1842,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>49.28</t>
+          <t>265.300401</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1867,12 +1859,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x060bae1553ca0b1b27e0303f5cb0b1a208018b22ad43c47887b7eab9174eb11f</t>
+          <t>0x798a2a121340304c054e489a82c2fbcbbacbb2b5a10fac5eccae9d0e6f953242</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x1EEc232fcA954D560922A46C0dc77A1d5Fc1278C</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1882,12 +1874,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.49999</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.7588</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1952,7 +1944,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786700992</t>
+          <t>1786704771</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1962,7 +1954,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.976923</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1979,7 +1971,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x89945f48362d177a1a075c347f0cee9e0d2949251232062e79954c3fdbda8548</t>
+          <t>0xd7c7ed5aee6d42691c0cdba24cc2a4844a2148619b251e896e222af12c3f399a</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1994,12 +1986,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>36.69</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.7475</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2064,7 +2056,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786697954</t>
+          <t>1786704503</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2074,7 +2066,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>49.083612</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2091,7 +2083,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x93f8ae4db5435f2088469fb82cd900c151ecf6b1707f1fa749e6f328a01576ca</t>
+          <t>0x91957fcc3f4e1390d64a84f24cad4ac44f2f9926c17ed7cd978de77f93ab840a</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2106,7 +2098,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>35.77998</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2176,7 +2168,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786696250</t>
+          <t>1786704472</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2186,7 +2178,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>47.70664</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2203,12 +2195,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x6c37a9cb7783035c2363518b021ca262c492e837d2f5566a7197ec81c9c7de3c</t>
+          <t>0x33ec03964bc9b5353ad6c834080797ae574d6738a2f6ecafd9040ba4d9dc21d6</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x2Bd56fa0D7b1Add3639Ee23f32A2947576924f15</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2218,22 +2210,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>557.83</t>
+          <t>36.96</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2258,7 +2250,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2288,7 +2280,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786696222</t>
+          <t>1786704050</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2298,7 +2290,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1025.894253</t>
+          <t>49.28</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2315,12 +2307,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xb8844dc9cad239dda58468ea8057a5d42a49adaeb39f853d1d8a2f72f86b2a27</t>
+          <t>0x060bae1553ca0b1b27e0303f5cb0b1a208018b22ad43c47887b7eab9174eb11f</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x1EEc232fcA954D560922A46C0dc77A1d5Fc1278C</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2330,22 +2322,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>22.83999</t>
+          <t>1.49999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.7588</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2370,7 +2362,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2400,7 +2392,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786695902</t>
+          <t>1786700992</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2410,7 +2402,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>42.004579</t>
+          <t>1.976923</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2427,7 +2419,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x54732df74313495ae4750f10f2ec1b1437622f274d00a56e3a61e0c23a1acde2</t>
+          <t>0x89945f48362d177a1a075c347f0cee9e0d2949251232062e79954c3fdbda8548</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2435,23 +2427,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>296.6897</t>
+          <t>36.69</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4612</t>
+          <t>1.7475</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786695873</t>
+          <t>1786697954</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>643.229702</t>
+          <t>49.083612</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2531,12 +2531,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x6388d0dbf04f19becbc0ad458a4000da4d11cf0c26aa897bddfdef754fa335a6</t>
+          <t>0x93f8ae4db5435f2088469fb82cd900c151ecf6b1707f1fa749e6f328a01576ca</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2546,22 +2546,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>346.54</t>
+          <t>35.77998</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786695869</t>
+          <t>1786696250</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>641.740741</t>
+          <t>47.70664</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2643,12 +2643,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x1d90dd2b57deb4a163be22ec0027c40ec930edc46ca3efc1b7765006d5e9eebe</t>
+          <t>0x6c37a9cb7783035c2363518b021ca262c492e837d2f5566a7197ec81c9c7de3c</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0x2Bd56fa0D7b1Add3639Ee23f32A2947576924f15</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2658,12 +2658,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>557.83</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786695799</t>
+          <t>1786696222</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.851852</t>
+          <t>1025.894253</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2755,12 +2755,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x48c4a72e45740310d60b3a648deeb512824e451ea186d1e82f9627f5d1bccd51</t>
+          <t>0xb8844dc9cad239dda58468ea8057a5d42a49adaeb39f853d1d8a2f72f86b2a27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2770,22 +2770,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.99999</t>
+          <t>22.83999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>LASK Linz -1</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786695700</t>
+          <t>1786695902</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1.33332</t>
+          <t>42.004579</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2867,27 +2867,23 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x4ebc4769fdeafa179bcff07b1f83a83c2f713dd0b038325187723d036f03b296</t>
+          <t>0x54732df74313495ae4750f10f2ec1b1437622f274d00a56e3a61e0c23a1acde2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0x9E555D159D333EAE7346aE58D3d57dDE9680a9F7</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>484.79999</t>
+          <t>296.6897</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.4612</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2895,11 +2891,7 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>LASK Linz -1</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -2952,7 +2944,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786695653</t>
+          <t>1786695873</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2962,7 +2954,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>897.777759</t>
+          <t>643.229702</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2979,12 +2971,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xb62e61543153c0b9ab6a1a3fd388b5a709ce3356240d5f06b0b8a0c62bad8b1a</t>
+          <t>0x6388d0dbf04f19becbc0ad458a4000da4d11cf0c26aa897bddfdef754fa335a6</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0x4c67719710F563c9CE4Df1836c8d643BACc6986a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2994,7 +2986,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>346.54</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3064,7 +3056,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786695037</t>
+          <t>1786695869</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3074,7 +3066,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>641.740741</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3091,12 +3083,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0xcb685b4fae14c825bf9607310b4cfb4892294304396aedd620dbe8ca7410b54c</t>
+          <t>0x1d90dd2b57deb4a163be22ec0027c40ec930edc46ca3efc1b7765006d5e9eebe</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3106,7 +3098,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3176,7 +3168,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786694953</t>
+          <t>1786695799</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3186,7 +3178,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>1.851852</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3203,12 +3195,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xbd2bb212ebdbf36503fd81ffa846a8c770a6aae66b0380af0fcc4a45aa66cc55</t>
+          <t>0x48c4a72e45740310d60b3a648deeb512824e451ea186d1e82f9627f5d1bccd51</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3218,22 +3210,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>0.99999</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>LASK Linz -1</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3258,7 +3250,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+          <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3288,7 +3280,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786694900</t>
+          <t>1786695700</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3298,7 +3290,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>555.555556</t>
+          <t>1.33332</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3315,23 +3307,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+          <t>0x4ebc4769fdeafa179bcff07b1f83a83c2f713dd0b038325187723d036f03b296</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>0x9E555D159D333EAE7346aE58D3d57dDE9680a9F7</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>23.34</t>
+          <t>484.79999</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.4638</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3339,7 +3335,11 @@
           <t>Asian Handicap (-1)</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>Bundesliga</t>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786682534</t>
+          <t>1786695653</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>50.328841</t>
+          <t>897.777759</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3419,102 +3419,542 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>0xb62e61543153c0b9ab6a1a3fd388b5a709ce3356240d5f06b0b8a0c62bad8b1a</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786695037</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0xcb685b4fae14c825bf9607310b4cfb4892294304396aedd620dbe8ca7410b54c</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786694953</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0xbd2bb212ebdbf36503fd81ffa846a8c770a6aae66b0380af0fcc4a45aa66cc55</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>LASK Linz -1</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1786694900</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>555.555556</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x9a4c9495704ee89e4ba79b9b36a31528db556fff6ab2c9dc478536c1cfb4c025</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>23.34</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4638</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Bundesliga</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LASK Linz vs SV Ried</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>LASK Linz</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>SV Ried</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0x01fc28e4c05acb8383b677e0a4bb44b143f7f41bef6d4a5a65902c464ac1e8d9</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19722986</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1786682534</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1786728600</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>50.328841</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>0xbc3f9a4aae23f8578c48b6575d84b3634a2c81e75a2b7c12b7aa17d431671a0e</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
         <is>
           <t>2.08</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>1.2625</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Under/Over (2)</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
         <is>
           <t>Bundesliga</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>LASK Linz vs SV Ried</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>LASK Linz</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>SV Ried</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>0x0f99df90038c8a3c1e5030e6029938911a2c71ab0d65fac4b3536f297fc63cbc</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>L19722986</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
         <is>
           <t>1786678003</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="S32" t="inlineStr">
         <is>
           <t>1786728600</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T32" t="inlineStr">
         <is>
           <t>7.92381</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>